<commit_message>
run 2019 for comparison
</commit_message>
<xml_diff>
--- a/01_data/02_output_data/02_unidirectional_results/02_paper_ESR/01_raw_results/outputs_ESR_2026_run_2019.xlsx
+++ b/01_data/02_output_data/02_unidirectional_results/02_paper_ESR/01_raw_results/outputs_ESR_2026_run_2019.xlsx
@@ -617,7 +617,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>517923.1571476575</v>
+        <v>443206.8863386028</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>309864.0358134354</v>
+        <v>235147.7650043806</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
@@ -905,7 +905,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>816050.2195434923</v>
+        <v>741333.9487344376</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>
@@ -929,7 +929,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>94759.02203752627</v>
+        <v>169475.292846581</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
@@ -1049,7 +1049,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>132064.8002240817</v>
+        <v>206781.0710331364</v>
       </c>
       <c r="D26" t="n">
         <v>0</v>
@@ -1121,7 +1121,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>18709.34182489541</v>
+        <v>93425.61263395014</v>
       </c>
       <c r="D29" t="n">
         <v>0</v>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>123041.5</v>
+        <v>73638.94582700002</v>
       </c>
       <c r="D34" t="n">
         <v>0</v>
@@ -1361,7 +1361,7 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>114026.8983795503</v>
+        <v>64624.34420655029</v>
       </c>
       <c r="D39" t="n">
         <v>0</v>
@@ -1505,7 +1505,7 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>202685.7237785689</v>
+        <v>127969.4529695142</v>
       </c>
       <c r="D45" t="n">
         <v>0</v>
@@ -1529,7 +1529,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>152659.350423</v>
+        <v>212659.350423</v>
       </c>
       <c r="D46" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>60000</v>
+        <v>74716.27080905481</v>
       </c>
       <c r="D53" t="n">
         <v>0</v>
@@ -1706,7 +1706,7 @@
         <v>1</v>
       </c>
       <c r="F53" t="n">
-        <v>60000</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="54">
@@ -2297,7 +2297,7 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>120000</v>
+        <v>180000</v>
       </c>
       <c r="D78" t="n">
         <v>0</v>
@@ -2306,7 +2306,7 @@
         <v>1</v>
       </c>
       <c r="F78" t="n">
-        <v>120000</v>
+        <v>180000</v>
       </c>
     </row>
     <row r="79">
@@ -2489,7 +2489,7 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>167406.5707137843</v>
+        <v>242122.841522839</v>
       </c>
       <c r="D86" t="n">
         <v>0</v>
@@ -2633,7 +2633,7 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>354643.730910441</v>
+        <v>429360.0017194957</v>
       </c>
       <c r="D92" t="n">
         <v>0</v>
@@ -2657,7 +2657,7 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>94243.41938852618</v>
+        <v>168959.6901975809</v>
       </c>
       <c r="D93" t="n">
         <v>0</v>
@@ -2873,7 +2873,7 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>392923.5512159909</v>
+        <v>318207.2804069361</v>
       </c>
       <c r="D102" t="n">
         <v>0</v>
@@ -3137,7 +3137,7 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>288731.64065</v>
+        <v>261991.64065</v>
       </c>
       <c r="D113" t="n">
         <v>0</v>
@@ -3185,7 +3185,7 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>122557.6514777237</v>
+        <v>47841.38066866901</v>
       </c>
       <c r="D115" t="n">
         <v>0</v>
@@ -3209,7 +3209,7 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>113102.8049452497</v>
+        <v>162505.3591182497</v>
       </c>
       <c r="D116" t="n">
         <v>0</v>
@@ -3665,7 +3665,7 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>573792.2721949819</v>
+        <v>521738.5555589272</v>
       </c>
       <c r="D135" t="n">
         <v>0</v>
@@ -3905,7 +3905,7 @@
         </is>
       </c>
       <c r="C145" t="n">
-        <v>73260</v>
+        <v>99999.99999999994</v>
       </c>
       <c r="D145" t="n">
         <v>0</v>
@@ -3914,7 +3914,7 @@
         <v>1</v>
       </c>
       <c r="F145" t="n">
-        <v>73260</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="146">
@@ -4409,7 +4409,7 @@
         </is>
       </c>
       <c r="C166" t="n">
-        <v>113102.8049452497</v>
+        <v>162505.3591182497</v>
       </c>
       <c r="D166" t="n">
         <v>0</v>
@@ -4553,7 +4553,7 @@
         </is>
       </c>
       <c r="C172" t="n">
-        <v>606521.0782649225</v>
+        <v>565161.7931158853</v>
       </c>
       <c r="D172" t="n">
         <v>0</v>
@@ -4745,7 +4745,7 @@
         </is>
       </c>
       <c r="C180" t="n">
-        <v>0</v>
+        <v>41359.28514903714</v>
       </c>
       <c r="D180" t="n">
         <v>0</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C202" t="n">
-        <v>78976.15878026752</v>
+        <v>29573.60460726754</v>
       </c>
       <c r="D202" t="n">
         <v>0</v>
@@ -6065,7 +6065,7 @@
         </is>
       </c>
       <c r="C235" t="n">
-        <v>122557.6514777237</v>
+        <v>47841.38066866901</v>
       </c>
       <c r="D235" t="n">
         <v>0</v>
@@ -6281,7 +6281,7 @@
         </is>
       </c>
       <c r="C244" t="n">
-        <v>455299.6498724489</v>
+        <v>507353.3665085036</v>
       </c>
       <c r="D244" t="n">
         <v>0</v>
@@ -6425,7 +6425,7 @@
         </is>
       </c>
       <c r="C250" t="n">
-        <v>59834.77695751414</v>
+        <v>82497.33113051415</v>
       </c>
       <c r="D250" t="n">
         <v>0</v>
@@ -6761,7 +6761,7 @@
         </is>
       </c>
       <c r="C264" t="n">
-        <v>10694.43148701754</v>
+        <v>0</v>
       </c>
       <c r="D264" t="n">
         <v>0</v>
@@ -6977,7 +6977,7 @@
         </is>
       </c>
       <c r="C273" t="n">
-        <v>563097.8407079644</v>
+        <v>521738.5555589272</v>
       </c>
       <c r="D273" t="n">
         <v>0</v>
@@ -7865,7 +7865,7 @@
         </is>
       </c>
       <c r="C310" t="n">
-        <v>838926.0366730001</v>
+        <v>849523.4825</v>
       </c>
       <c r="D310" t="n">
         <v>0</v>
@@ -8297,7 +8297,7 @@
         </is>
       </c>
       <c r="C328" t="n">
-        <v>142068</v>
+        <v>156784.2708090548</v>
       </c>
       <c r="D328" t="n">
         <v>0</v>
@@ -8969,7 +8969,7 @@
         </is>
       </c>
       <c r="C356" t="n">
-        <v>1004229.551874768</v>
+        <v>952175.8352387138</v>
       </c>
       <c r="D356" t="n">
         <v>0</v>
@@ -9089,7 +9089,7 @@
         </is>
       </c>
       <c r="C361" t="n">
-        <v>1493732.579193929</v>
+        <v>1520472.579193929</v>
       </c>
       <c r="D361" t="n">
         <v>0</v>
@@ -17993,10 +17993,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>517923.1571476575</v>
+        <v>443206.8863386028</v>
       </c>
       <c r="D8" t="n">
-        <v>0.6230099902657177</v>
+        <v>0.5331337557181108</v>
       </c>
     </row>
     <row r="9">
@@ -18047,10 +18047,10 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>309864.0358134354</v>
+        <v>235147.7650043806</v>
       </c>
       <c r="D11" t="n">
-        <v>0.7389820367970281</v>
+        <v>0.5607942653784787</v>
       </c>
     </row>
     <row r="12">
@@ -18209,10 +18209,10 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>816050.2195434923</v>
+        <v>741333.9487344376</v>
       </c>
       <c r="D20" t="n">
-        <v>0.4095155970280194</v>
+        <v>0.3720209949615023</v>
       </c>
     </row>
     <row r="21">
@@ -18227,10 +18227,10 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>94759.02203752627</v>
+        <v>169475.292846581</v>
       </c>
       <c r="D21" t="n">
-        <v>0.3054279517728486</v>
+        <v>0.5462539656618243</v>
       </c>
     </row>
     <row r="22">
@@ -18317,10 +18317,10 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>132064.8002240817</v>
+        <v>206781.0710331364</v>
       </c>
       <c r="D26" t="n">
-        <v>0.3754891765015941</v>
+        <v>0.5879239127050285</v>
       </c>
     </row>
     <row r="27">
@@ -18371,10 +18371,10 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>18709.34182489541</v>
+        <v>93425.61263395014</v>
       </c>
       <c r="D29" t="n">
-        <v>0.05502197375819892</v>
+        <v>0.2747537382554396</v>
       </c>
     </row>
     <row r="30">
@@ -18461,10 +18461,10 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>123041.5</v>
+        <v>73638.94582700002</v>
       </c>
       <c r="D34" t="n">
-        <v>1</v>
+        <v>0.5984886873697087</v>
       </c>
     </row>
     <row r="35">
@@ -18551,10 +18551,10 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>114026.8983795503</v>
+        <v>64624.34420655029</v>
       </c>
       <c r="D39" t="n">
-        <v>0.7055159469598834</v>
+        <v>0.3998486852442755</v>
       </c>
     </row>
     <row r="40">
@@ -18659,10 +18659,10 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>202685.7237785689</v>
+        <v>127969.4529695142</v>
       </c>
       <c r="D45" t="n">
-        <v>0.2916114060269128</v>
+        <v>0.1841143589851625</v>
       </c>
     </row>
     <row r="46">
@@ -18677,10 +18677,10 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>152659.350423</v>
+        <v>212659.350423</v>
       </c>
       <c r="D46" t="n">
-        <v>0.3624304988556777</v>
+        <v>0.5048772593789321</v>
       </c>
     </row>
     <row r="47">
@@ -18803,10 +18803,10 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>60000</v>
+        <v>74716.27080905481</v>
       </c>
       <c r="D53" t="n">
-        <v>1</v>
+        <v>0.7471627080905481</v>
       </c>
     </row>
     <row r="54">
@@ -19253,7 +19253,7 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>120000</v>
+        <v>180000</v>
       </c>
       <c r="D78" t="n">
         <v>1</v>
@@ -19397,10 +19397,10 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>167406.5707137843</v>
+        <v>242122.841522839</v>
       </c>
       <c r="D86" t="n">
-        <v>0.3819839584757849</v>
+        <v>0.5524696016886019</v>
       </c>
     </row>
     <row r="87">
@@ -19505,10 +19505,10 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>354643.730910441</v>
+        <v>429360.0017194957</v>
       </c>
       <c r="D92" t="n">
-        <v>0.809216840200388</v>
+        <v>0.979702483413205</v>
       </c>
     </row>
     <row r="93">
@@ -19523,10 +19523,10 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>94243.41938852618</v>
+        <v>168959.6901975809</v>
       </c>
       <c r="D93" t="n">
-        <v>0.1797017237272181</v>
+        <v>0.322169417938358</v>
       </c>
     </row>
     <row r="94">
@@ -19685,10 +19685,10 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>392923.5512159909</v>
+        <v>318207.2804069361</v>
       </c>
       <c r="D102" t="n">
-        <v>0.6300128050821154</v>
+        <v>0.5102128918114245</v>
       </c>
     </row>
     <row r="103">
@@ -19883,10 +19883,10 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>288731.64065</v>
+        <v>261991.64065</v>
       </c>
       <c r="D113" t="n">
-        <v>0.6778183557839482</v>
+        <v>0.6150442767364992</v>
       </c>
     </row>
     <row r="114">
@@ -19919,10 +19919,10 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>122557.6514777237</v>
+        <v>47841.38066866901</v>
       </c>
       <c r="D115" t="n">
-        <v>0.3801298082495077</v>
+        <v>0.1483867766777365</v>
       </c>
     </row>
     <row r="116">
@@ -19937,10 +19937,10 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>113102.8049452497</v>
+        <v>162505.3591182497</v>
       </c>
       <c r="D116" t="n">
-        <v>0.1926213134118839</v>
+        <v>0.2767570240630163</v>
       </c>
     </row>
     <row r="117">
@@ -20279,10 +20279,10 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>573792.2721949819</v>
+        <v>521738.5555589272</v>
       </c>
       <c r="D135" t="n">
-        <v>0.0005737922727687742</v>
+        <v>0.0005217385560806658</v>
       </c>
     </row>
     <row r="136">
@@ -20459,10 +20459,10 @@
         </is>
       </c>
       <c r="C145" t="n">
-        <v>73260</v>
+        <v>99999.99999999994</v>
       </c>
       <c r="D145" t="n">
-        <v>1</v>
+        <v>0.9999999999999994</v>
       </c>
     </row>
     <row r="146">
@@ -20837,10 +20837,10 @@
         </is>
       </c>
       <c r="C166" t="n">
-        <v>113102.8049452497</v>
+        <v>162505.3591182497</v>
       </c>
       <c r="D166" t="n">
-        <v>0.0001131028050583525</v>
+        <v>0.000162505359280755</v>
       </c>
     </row>
     <row r="167">
@@ -20945,10 +20945,10 @@
         </is>
       </c>
       <c r="C172" t="n">
-        <v>606521.0782649225</v>
+        <v>565161.7931158853</v>
       </c>
       <c r="D172" t="n">
-        <v>0.0006065210788714436</v>
+        <v>0.0005651617936810471</v>
       </c>
     </row>
     <row r="173">
@@ -21089,10 +21089,10 @@
         </is>
       </c>
       <c r="C180" t="n">
-        <v>0</v>
+        <v>41359.28514903714</v>
       </c>
       <c r="D180" t="n">
-        <v>0</v>
+        <v>4.135928519039643e-05</v>
       </c>
     </row>
     <row r="181">
@@ -21485,10 +21485,10 @@
         </is>
       </c>
       <c r="C202" t="n">
-        <v>78976.15878026752</v>
+        <v>29573.60460726754</v>
       </c>
       <c r="D202" t="n">
-        <v>7.897615885924368e-05</v>
+        <v>2.957360463684114e-05</v>
       </c>
     </row>
     <row r="203">
@@ -22079,10 +22079,10 @@
         </is>
       </c>
       <c r="C235" t="n">
-        <v>122557.6514777237</v>
+        <v>47841.38066866901</v>
       </c>
       <c r="D235" t="n">
-        <v>0.0001225576516002814</v>
+        <v>4.784138071651039e-05</v>
       </c>
     </row>
     <row r="236">
@@ -22241,10 +22241,10 @@
         </is>
       </c>
       <c r="C244" t="n">
-        <v>455299.6498724489</v>
+        <v>507353.3665085036</v>
       </c>
       <c r="D244" t="n">
-        <v>0.0004552996503277485</v>
+        <v>0.0005073533670158569</v>
       </c>
     </row>
     <row r="245">
@@ -22349,10 +22349,10 @@
         </is>
       </c>
       <c r="C250" t="n">
-        <v>59834.77695751414</v>
+        <v>82497.33113051415</v>
       </c>
       <c r="D250" t="n">
-        <v>5.983477701734892e-05</v>
+        <v>8.249733121301149e-05</v>
       </c>
     </row>
     <row r="251">
@@ -22601,10 +22601,10 @@
         </is>
       </c>
       <c r="C264" t="n">
-        <v>10694.43148701754</v>
+        <v>0</v>
       </c>
       <c r="D264" t="n">
-        <v>1.069443149771198e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="265">
@@ -22763,10 +22763,10 @@
         </is>
       </c>
       <c r="C273" t="n">
-        <v>563097.8407079644</v>
+        <v>521738.5555589272</v>
       </c>
       <c r="D273" t="n">
-        <v>0.0005630978412710622</v>
+        <v>0.0005217385560806658</v>
       </c>
     </row>
     <row r="274">
@@ -23429,10 +23429,10 @@
         </is>
       </c>
       <c r="C310" t="n">
-        <v>838926.0366730001</v>
+        <v>849523.4825</v>
       </c>
       <c r="D310" t="n">
-        <v>0.0008389260375119261</v>
+        <v>0.0008495234833495235</v>
       </c>
     </row>
     <row r="311">
@@ -23753,10 +23753,10 @@
         </is>
       </c>
       <c r="C328" t="n">
-        <v>142068</v>
+        <v>156784.2708090548</v>
       </c>
       <c r="D328" t="n">
-        <v>0.000142068000142068</v>
+        <v>0.0001567842709658391</v>
       </c>
     </row>
     <row r="329">
@@ -24257,10 +24257,10 @@
         </is>
       </c>
       <c r="C356" t="n">
-        <v>1004229.551874768</v>
+        <v>952175.8352387138</v>
       </c>
       <c r="D356" t="n">
-        <v>0.001004229552878998</v>
+        <v>0.0009521758361908896</v>
       </c>
     </row>
     <row r="357">
@@ -24347,10 +24347,10 @@
         </is>
       </c>
       <c r="C361" t="n">
-        <v>1493732.579193929</v>
+        <v>1520472.579193929</v>
       </c>
       <c r="D361" t="n">
-        <v>0.001493732580687661</v>
+        <v>0.001520472580714401</v>
       </c>
     </row>
     <row r="362">

</xml_diff>